<commit_message>
fix(documents): RO_CIPL / con_CIPL 파일 손상 — 외부 참조 definedName 50+개 제거
증상: 생성된 .xlsx를 Excel에서 열면 "파일 손상" 에러 또는 복구 모드 진입.

원인: 원본 xlsm에서 시트만 추출했지만 워크북 레벨 `<definedName>`(외부
워크북 [1]/[3]/[4]/[7] 등으로의 참조 + 본 시트의 #REF! 잘못된 정의)이
50+개 그대로 남아있었음. Excel이 깨진 외부 참조를 만나 손상으로 판단.

수정: 템플릿 추출 단계에서 wb.defined_names 비움 + ws.defined_names 비움.
표준 Print_Titles / Print_Area 2개만 유지 (페이지 출력에 필요).

검증: openpyxl 경고 없이 로드 / definedName 50+ → 2 / 파일 사이즈 90KB → 71KB.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/templates/con_cipl_template.xlsx
+++ b/resources/templates/con_cipl_template.xlsx
@@ -8,123 +8,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="con_CIPL" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
-  </externalReferences>
   <definedNames>
-    <definedName name="AA">[1]입출고!#REF!</definedName>
-    <definedName name="GG">#REF!</definedName>
-    <definedName name="ID">[4]입출고!#REF!</definedName>
-    <definedName name="YY">'[5]1'!#REF!</definedName>
-    <definedName name="계산서">[4]입출고!#REF!</definedName>
-    <definedName name="계약금">[4]입출고!#REF!</definedName>
-    <definedName name="광택">[4]입출고!#REF!</definedName>
-    <definedName name="구분입력">[7]수출현황_종합!$G$2</definedName>
-    <definedName name="구분입력2">[7]수출현황_종합!$G$3</definedName>
-    <definedName name="기준날짜">[7]수출현황_종합!$J$3</definedName>
-    <definedName name="기준월">[7]수출현황_종합!$C$3</definedName>
-    <definedName name="기타">[4]입출고!#REF!</definedName>
-    <definedName name="ㄴㅇㄹ">'[8]1'!#REF!</definedName>
-    <definedName name="년도">[7]수출현황_종합!$B$3</definedName>
-    <definedName name="등급">[4]입출고!#REF!</definedName>
-    <definedName name="말소날짜">[4]입출고!#REF!</definedName>
-    <definedName name="매입가">[4]입출고!#REF!</definedName>
-    <definedName name="매입날짜">[4]입출고!#REF!</definedName>
-    <definedName name="메다">[4]입출고!#REF!</definedName>
-    <definedName name="미수">[4]입출고!#REF!</definedName>
-    <definedName name="바이어연락처">[4]입출고!#REF!</definedName>
-    <definedName name="변속기">[4]입출고!#REF!</definedName>
-    <definedName name="ㅅ">'[8]1'!#REF!</definedName>
-    <definedName name="사업자">[4]입출고!#REF!</definedName>
-    <definedName name="사진">[4]입출고!#REF!</definedName>
-    <definedName name="색상">[4]입출고!#REF!</definedName>
-    <definedName name="선적계획">[4]입출고!#REF!</definedName>
-    <definedName name="수출종합" hidden="1">[7]수출현황_종합!$B$12:$AL$15</definedName>
-    <definedName name="쉬핑오더">#REF!</definedName>
-    <definedName name="시스템">[4]입출고!#REF!</definedName>
-    <definedName name="시트">[4]입출고!#REF!</definedName>
-    <definedName name="실매입가">[4]입출고!#REF!</definedName>
-    <definedName name="업체">#REF!</definedName>
-    <definedName name="연식">[4]입출고!#REF!</definedName>
-    <definedName name="운임">[4]입출고!#REF!</definedName>
-    <definedName name="월">[7]수출현황_종합!$J$4</definedName>
-    <definedName name="유리">[4]입출고!#REF!</definedName>
-    <definedName name="잔금">[4]입출고!#REF!</definedName>
-    <definedName name="재고">[4]입출고!#REF!</definedName>
-    <definedName name="정비수리">[4]입출고!#REF!</definedName>
-    <definedName name="조건범위">#REF!</definedName>
-    <definedName name="주민번호">[4]입출고!#REF!</definedName>
-    <definedName name="주소">[4]입출고!#REF!</definedName>
-    <definedName name="주행거리">[4]입출고!#REF!</definedName>
-    <definedName name="ㅊ">'[8]1'!#REF!</definedName>
-    <definedName name="차대번호">[4]입출고!#REF!</definedName>
-    <definedName name="차량명">[4]입출고!#REF!</definedName>
-    <definedName name="차량번호">[4]입출고!#REF!</definedName>
-    <definedName name="차명">[7]CarName_INPUT입력!$A$4:$A$423</definedName>
-    <definedName name="차주">[4]입출고!#REF!</definedName>
-    <definedName name="차주연락처">[4]입출고!#REF!</definedName>
-    <definedName name="출력범위">#REF!</definedName>
-    <definedName name="판금도색">[4]입출고!#REF!</definedName>
-    <definedName name="판매가">[4]입출고!#REF!</definedName>
-    <definedName name="판매바이어">[4]입출고!#REF!</definedName>
-    <definedName name="GG" localSheetId="0">con_CIPL!#REF!</definedName>
-    <definedName name="ID" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="YY" localSheetId="0">'[5]1'!#REF!</definedName>
-    <definedName name="계산서" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="계약금" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="광택" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="구분입력" localSheetId="0">[6]수출현황_종합!$G$2</definedName>
-    <definedName name="구분입력2" localSheetId="0">[6]수출현황_종합!$G$3</definedName>
-    <definedName name="기준날짜" localSheetId="0">[6]수출현황_종합!$J$3</definedName>
-    <definedName name="기준월" localSheetId="0">[6]수출현황_종합!$C$3</definedName>
-    <definedName name="기타" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="ㄴㅇㄹ" localSheetId="0">'[8]1'!#REF!</definedName>
-    <definedName name="년도" localSheetId="0">[6]수출현황_종합!$B$3</definedName>
-    <definedName name="등급" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="말소날짜" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="매입가" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="매입날짜" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="메다" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="미수" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="바이어연락처" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="변속기" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="사업자" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="사진" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="색상" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="선적계획" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="수출종합" localSheetId="0" hidden="1">[6]수출현황_종합!$B$12:$AL$15</definedName>
-    <definedName name="쉬핑오더" localSheetId="0">con_CIPL!#REF!</definedName>
-    <definedName name="시스템" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="시트" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="실매입가" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="연식" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="운임" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="월" localSheetId="0">[6]수출현황_종합!$J$4</definedName>
-    <definedName name="유리" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="잔금" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="재고" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="정비수리" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="주민번호" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="주소" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="주행거리" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="ㅊ" localSheetId="0">'[8]1'!#REF!</definedName>
-    <definedName name="차대번호" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="차량명" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="차량번호" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="차명" localSheetId="0">[9]CarName_INPUT입력!$A$4:$A$423</definedName>
-    <definedName name="차주" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="차주연락처" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="판금도색" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="판매가" localSheetId="0">[3]입출고!#REF!</definedName>
-    <definedName name="판매바이어" localSheetId="0">[3]입출고!#REF!</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'con_CIPL'!$20:$20</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'con_CIPL'!$B$1:$L$46</definedName>
   </definedNames>
@@ -19927,4701 +19811,6 @@
     <clientData/>
   </twoCellAnchor>
 </wsDr>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="입출고"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="입출고"/>
-      <sheetName val="차량말소신청서"/>
-      <sheetName val="2.계약서"/>
-      <sheetName val="사업자"/>
-      <sheetName val="등기부등본"/>
-      <sheetName val="법인대표 신분증"/>
-      <sheetName val="관련서류"/>
-      <sheetName val="매매계약서 수출용"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="현황판"/>
-      <sheetName val="입출고"/>
-      <sheetName val="차량말소신청서"/>
-      <sheetName val="사업자등록증"/>
-      <sheetName val="계약서"/>
-      <sheetName val="매매계약서"/>
-      <sheetName val="매매계약서 수출용"/>
-      <sheetName val="2016 년도 성신무역 현황표"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="현황판"/>
-      <sheetName val="입출고"/>
-      <sheetName val="차량말소신청서"/>
-      <sheetName val="사업자등록증"/>
-      <sheetName val="계약서"/>
-      <sheetName val="매매계약서"/>
-      <sheetName val="매매계약서 수출용"/>
-      <sheetName val="2016 년도 성신무역 현황표"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink5.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="12 (3)"/>
-      <sheetName val="1"/>
-      <sheetName val="1(2)"/>
-      <sheetName val="2"/>
-      <sheetName val="2 (2)"/>
-      <sheetName val="3"/>
-      <sheetName val="3(2)"/>
-      <sheetName val="4"/>
-      <sheetName val="4 (2)"/>
-      <sheetName val="5"/>
-      <sheetName val="5 (2)"/>
-      <sheetName val="6"/>
-      <sheetName val="6 (2)"/>
-      <sheetName val="7"/>
-      <sheetName val="7 (2)"/>
-      <sheetName val="8"/>
-      <sheetName val="8 (2)"/>
-      <sheetName val="9"/>
-      <sheetName val="9 (2)"/>
-      <sheetName val="10"/>
-      <sheetName val="10 (2)"/>
-      <sheetName val="11"/>
-      <sheetName val="11 (2)"/>
-      <sheetName val="12"/>
-      <sheetName val="12 (2)"/>
-      <sheetName val="집계표"/>
-      <sheetName val="잔액"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13" refreshError="1"/>
-      <sheetData sheetId="14" refreshError="1"/>
-      <sheetData sheetId="15" refreshError="1"/>
-      <sheetData sheetId="16" refreshError="1"/>
-      <sheetData sheetId="17" refreshError="1"/>
-      <sheetData sheetId="18" refreshError="1"/>
-      <sheetData sheetId="19" refreshError="1"/>
-      <sheetData sheetId="20" refreshError="1"/>
-      <sheetData sheetId="21" refreshError="1"/>
-      <sheetData sheetId="22" refreshError="1"/>
-      <sheetData sheetId="23" refreshError="1"/>
-      <sheetData sheetId="24"/>
-      <sheetData sheetId="25" refreshError="1"/>
-      <sheetData sheetId="26" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink6.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="20161130이후"/>
-      <sheetName val="CarName_INPUT입력"/>
-      <sheetName val="쉬핑마크 (2)"/>
-      <sheetName val="쉬핑마크"/>
-      <sheetName val="계약서"/>
-      <sheetName val="쉬핑INVOICE"/>
-      <sheetName val="수출현황_종합"/>
-      <sheetName val="부품"/>
-      <sheetName val="차량매입경비신청서 (2)"/>
-      <sheetName val="신한 원화"/>
-      <sheetName val="코리아 원화"/>
-      <sheetName val="차량매입경비신청서"/>
-      <sheetName val="면장신청"/>
-      <sheetName val="Sheet2"/>
-      <sheetName val="Sheet3"/>
-      <sheetName val="말소신청서"/>
-      <sheetName val="월말신고"/>
-      <sheetName val="구매선적일보"/>
-      <sheetName val="매입현황 보고"/>
-      <sheetName val="재고관리"/>
-      <sheetName val="말소증"/>
-      <sheetName val="매매계약서"/>
-      <sheetName val="면장주소"/>
-      <sheetName val="현금영수증"/>
-      <sheetName val="이행신고서"/>
-      <sheetName val="개인정보"/>
-      <sheetName val="Sheet1"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>차명</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6">
-        <row r="2">
-          <cell r="G2" t="str">
-            <v>C142</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="B3">
-            <v>2017</v>
-          </cell>
-          <cell r="C3">
-            <v>5</v>
-          </cell>
-          <cell r="G3">
-            <v>0</v>
-          </cell>
-          <cell r="J3">
-            <v>42856</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="J4">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="B12">
-            <v>0</v>
-          </cell>
-          <cell r="C12">
-            <v>0</v>
-          </cell>
-          <cell r="D12">
-            <v>0</v>
-          </cell>
-          <cell r="E12">
-            <v>0</v>
-          </cell>
-          <cell r="F12">
-            <v>0</v>
-          </cell>
-          <cell r="G12">
-            <v>0</v>
-          </cell>
-          <cell r="H12">
-            <v>0</v>
-          </cell>
-          <cell r="I12">
-            <v>0</v>
-          </cell>
-          <cell r="J12">
-            <v>0</v>
-          </cell>
-          <cell r="K12">
-            <v>0</v>
-          </cell>
-          <cell r="L12">
-            <v>0</v>
-          </cell>
-          <cell r="M12">
-            <v>0</v>
-          </cell>
-          <cell r="N12">
-            <v>0</v>
-          </cell>
-          <cell r="Q12">
-            <v>0</v>
-          </cell>
-          <cell r="R12">
-            <v>0</v>
-          </cell>
-          <cell r="S12">
-            <v>0</v>
-          </cell>
-          <cell r="T12">
-            <v>29</v>
-          </cell>
-          <cell r="U12">
-            <v>0</v>
-          </cell>
-          <cell r="V12">
-            <v>0</v>
-          </cell>
-          <cell r="X12">
-            <v>0</v>
-          </cell>
-          <cell r="Y12">
-            <v>0</v>
-          </cell>
-          <cell r="Z12">
-            <v>0</v>
-          </cell>
-          <cell r="AB12">
-            <v>0</v>
-          </cell>
-          <cell r="AC12">
-            <v>0</v>
-          </cell>
-          <cell r="AD12">
-            <v>0</v>
-          </cell>
-          <cell r="AE12">
-            <v>0</v>
-          </cell>
-          <cell r="AF12">
-            <v>0</v>
-          </cell>
-          <cell r="AG12">
-            <v>0</v>
-          </cell>
-          <cell r="AH12">
-            <v>0</v>
-          </cell>
-          <cell r="AI12">
-            <v>0</v>
-          </cell>
-          <cell r="AJ12">
-            <v>0</v>
-          </cell>
-          <cell r="AK12">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="B13">
-            <v>0</v>
-          </cell>
-          <cell r="C13">
-            <v>0</v>
-          </cell>
-          <cell r="D13" t="str">
-            <v>매매계약서</v>
-          </cell>
-          <cell r="E13">
-            <v>0</v>
-          </cell>
-          <cell r="F13">
-            <v>0</v>
-          </cell>
-          <cell r="G13">
-            <v>0</v>
-          </cell>
-          <cell r="H13" t="str">
-            <v>재고</v>
-          </cell>
-          <cell r="I13">
-            <v>281</v>
-          </cell>
-          <cell r="J13">
-            <v>0</v>
-          </cell>
-          <cell r="K13">
-            <v>0</v>
-          </cell>
-          <cell r="L13">
-            <v>25</v>
-          </cell>
-          <cell r="M13">
-            <v>0</v>
-          </cell>
-          <cell r="N13">
-            <v>0</v>
-          </cell>
-          <cell r="Q13">
-            <v>0</v>
-          </cell>
-          <cell r="R13">
-            <v>0</v>
-          </cell>
-          <cell r="S13">
-            <v>0</v>
-          </cell>
-          <cell r="T13">
-            <v>0</v>
-          </cell>
-          <cell r="U13">
-            <v>0</v>
-          </cell>
-          <cell r="V13">
-            <v>0</v>
-          </cell>
-          <cell r="W13">
-            <v>0</v>
-          </cell>
-          <cell r="X13">
-            <v>0</v>
-          </cell>
-          <cell r="Y13">
-            <v>0</v>
-          </cell>
-          <cell r="Z13">
-            <v>0</v>
-          </cell>
-          <cell r="AB13">
-            <v>0</v>
-          </cell>
-          <cell r="AC13">
-            <v>0</v>
-          </cell>
-          <cell r="AD13">
-            <v>0</v>
-          </cell>
-          <cell r="AE13">
-            <v>0</v>
-          </cell>
-          <cell r="AF13">
-            <v>0</v>
-          </cell>
-          <cell r="AG13">
-            <v>0</v>
-          </cell>
-          <cell r="AH13">
-            <v>0</v>
-          </cell>
-          <cell r="AI13">
-            <v>0</v>
-          </cell>
-          <cell r="AJ13">
-            <v>0</v>
-          </cell>
-          <cell r="AK13">
-            <v>0</v>
-          </cell>
-          <cell r="AL13" t="str">
-            <v>전체</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="B14" t="str">
-            <v>구분입력</v>
-          </cell>
-          <cell r="C14" t="str">
-            <v>2회사</v>
-          </cell>
-          <cell r="D14" t="str">
-            <v>3번호</v>
-          </cell>
-          <cell r="E14" t="str">
-            <v>4날짜</v>
-          </cell>
-          <cell r="F14" t="str">
-            <v>5차번</v>
-          </cell>
-          <cell r="G14" t="str">
-            <v>6차명</v>
-          </cell>
-          <cell r="H14" t="str">
-            <v>7연식</v>
-          </cell>
-          <cell r="I14" t="str">
-            <v>8세금계산서</v>
-          </cell>
-          <cell r="J14" t="str">
-            <v>9면장액</v>
-          </cell>
-          <cell r="K14" t="str">
-            <v>10매입액</v>
-          </cell>
-          <cell r="L14" t="str">
-            <v>11등록번호</v>
-          </cell>
-          <cell r="M14" t="str">
-            <v>12매출일</v>
-          </cell>
-          <cell r="N14" t="str">
-            <v>13차대번호</v>
-          </cell>
-          <cell r="O14" t="str">
-            <v>14말소일</v>
-          </cell>
-          <cell r="P14" t="str">
-            <v>15관청</v>
-          </cell>
-          <cell r="Q14" t="str">
-            <v>16메모</v>
-          </cell>
-          <cell r="R14" t="str">
-            <v>17면장</v>
-          </cell>
-          <cell r="S14" t="str">
-            <v>18면장번호</v>
-          </cell>
-          <cell r="T14" t="str">
-            <v>선적
-업체20</v>
-          </cell>
-          <cell r="U14" t="str">
-            <v>b/l no.21</v>
-          </cell>
-          <cell r="V14" t="str">
-            <v>21색깔</v>
-          </cell>
-          <cell r="W14" t="str">
-            <v>도착지22</v>
-          </cell>
-          <cell r="X14" t="str">
-            <v>바이어23</v>
-          </cell>
-          <cell r="Y14" t="str">
-            <v>CONSIGNEE24</v>
-          </cell>
-          <cell r="Z14" t="str">
-            <v>팩스25</v>
-          </cell>
-          <cell r="AA14" t="str">
-            <v>바이어전화번호26</v>
-          </cell>
-          <cell r="AB14" t="str">
-            <v>판매금액27</v>
-          </cell>
-          <cell r="AC14" t="str">
-            <v>계약금28</v>
-          </cell>
-          <cell r="AD14" t="str">
-            <v>잔금29</v>
-          </cell>
-          <cell r="AE14" t="str">
-            <v>주행거리30</v>
-          </cell>
-          <cell r="AF14" t="str">
-            <v>사업자&amp;환급여부31</v>
-          </cell>
-          <cell r="AG14" t="str">
-            <v>수출이행32</v>
-          </cell>
-          <cell r="AH14" t="str">
-            <v>계산서/환급33</v>
-          </cell>
-          <cell r="AI14" t="str">
-            <v>차주성명34</v>
-          </cell>
-          <cell r="AJ14" t="str">
-            <v>주민등록번호35</v>
-          </cell>
-          <cell r="AK14" t="str">
-            <v>주소36</v>
-          </cell>
-          <cell r="AL14" t="str">
-            <v>성명37</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="B15">
-            <v>530</v>
-          </cell>
-          <cell r="C15" t="str">
-            <v>성신</v>
-          </cell>
-          <cell r="D15" t="str">
-            <v xml:space="preserve"> / No.1</v>
-          </cell>
-          <cell r="E15">
-            <v>42607</v>
-          </cell>
-          <cell r="F15" t="str">
-            <v>마티즈</v>
-          </cell>
-          <cell r="G15" t="str">
-            <v xml:space="preserve">DAEWOO  MATIZ </v>
-          </cell>
-          <cell r="H15" t="str">
-            <v>2001</v>
-          </cell>
-          <cell r="I15">
-            <v>0</v>
-          </cell>
-          <cell r="J15">
-            <v>0</v>
-          </cell>
-          <cell r="K15">
-            <v>0</v>
-          </cell>
-          <cell r="L15" t="str">
-            <v>17소8195</v>
-          </cell>
-          <cell r="M15">
-            <v>0</v>
-          </cell>
-          <cell r="N15" t="str">
-            <v>KLY4A11BD1C726117</v>
-          </cell>
-          <cell r="O15">
-            <v>42607</v>
-          </cell>
-          <cell r="P15" t="str">
-            <v>인천광역시 연수구청장</v>
-          </cell>
-          <cell r="Q15">
-            <v>0</v>
-          </cell>
-          <cell r="R15">
-            <v>42768</v>
-          </cell>
-          <cell r="S15">
-            <v>4374</v>
-          </cell>
-          <cell r="T15">
-            <v>0</v>
-          </cell>
-          <cell r="U15">
-            <v>0</v>
-          </cell>
-          <cell r="V15">
-            <v>0</v>
-          </cell>
-          <cell r="W15" t="str">
-            <v>UZB</v>
-          </cell>
-          <cell r="X15">
-            <v>0</v>
-          </cell>
-          <cell r="Y15">
-            <v>0</v>
-          </cell>
-          <cell r="Z15">
-            <v>0</v>
-          </cell>
-          <cell r="AA15">
-            <v>0</v>
-          </cell>
-          <cell r="AB15">
-            <v>0</v>
-          </cell>
-          <cell r="AC15">
-            <v>0</v>
-          </cell>
-          <cell r="AD15">
-            <v>0</v>
-          </cell>
-          <cell r="AE15">
-            <v>0</v>
-          </cell>
-          <cell r="AF15">
-            <v>0</v>
-          </cell>
-          <cell r="AG15">
-            <v>0</v>
-          </cell>
-          <cell r="AH15">
-            <v>0</v>
-          </cell>
-          <cell r="AI15">
-            <v>0</v>
-          </cell>
-          <cell r="AJ15">
-            <v>0</v>
-          </cell>
-          <cell r="AK15">
-            <v>0</v>
-          </cell>
-          <cell r="AL15">
-            <v>0</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-      <sheetData sheetId="21"/>
-      <sheetData sheetId="22"/>
-      <sheetData sheetId="23"/>
-      <sheetData sheetId="24"/>
-      <sheetData sheetId="25"/>
-      <sheetData sheetId="26"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink7.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="20161130이후"/>
-      <sheetName val="CarName_INPUT입력"/>
-      <sheetName val="쉬핑마크 (2)"/>
-      <sheetName val="쉬핑마크"/>
-      <sheetName val="계약서"/>
-      <sheetName val="쉬핑INVOICE"/>
-      <sheetName val="수출현황_종합"/>
-      <sheetName val="부품"/>
-      <sheetName val="차량매입경비신청서 (2)"/>
-      <sheetName val="신한 원화"/>
-      <sheetName val="코리아 원화"/>
-      <sheetName val="차량매입경비신청서"/>
-      <sheetName val="면장신청"/>
-      <sheetName val="Sheet2"/>
-      <sheetName val="Sheet3"/>
-      <sheetName val="말소신청서"/>
-      <sheetName val="월말신고"/>
-      <sheetName val="구매선적일보"/>
-      <sheetName val="매입현황 보고"/>
-      <sheetName val="재고관리"/>
-      <sheetName val="말소증"/>
-      <sheetName val="매매계약서"/>
-      <sheetName val="면장주소"/>
-      <sheetName val="현금영수증"/>
-      <sheetName val="이행신고서"/>
-      <sheetName val="개인정보"/>
-      <sheetName val="Sheet1"/>
-      <sheetName val="입출고"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>차명</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>엑센트1495</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>엑센트1396</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>엑센트1341</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8" t="str">
-            <v>엑센트1591</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9" t="str">
-            <v>엑센트1368</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10" t="str">
-            <v>엑센트1582</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11" t="str">
-            <v>엑센트</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12" t="str">
-            <v>아반떼</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13" t="str">
-            <v>md</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14" t="str">
-            <v>아반떼오토</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="A15" t="str">
-            <v>hd</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="A16" t="str">
-            <v>xd</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="A17" t="str">
-            <v>뉴아반떼</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="A18" t="str">
-            <v>클릭</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="A19" t="str">
-            <v>뉴클릭</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="A20" t="str">
-            <v>엘란트라</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="A21" t="str">
-            <v>그레이스</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="A22" t="str">
-            <v>그레이스9</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="A23" t="str">
-            <v>그레이스12</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="A24">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="A25" t="str">
-            <v>그레이스15</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="A26">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="A27" t="str">
-            <v>그레이스6밴</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="A28" t="str">
-            <v>그레이스
-장축6밴</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="A29" t="str">
-            <v>그레이스
-장축3밴</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="A30">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="A31" t="str">
-            <v>마이티 2.5톤</v>
-          </cell>
-        </row>
-        <row r="32">
-          <cell r="A32" t="str">
-            <v>마이티</v>
-          </cell>
-        </row>
-        <row r="33">
-          <cell r="A33" t="str">
-            <v>마이티2 터보</v>
-          </cell>
-        </row>
-        <row r="34">
-          <cell r="A34">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="35">
-          <cell r="A35">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="36">
-          <cell r="A36" t="str">
-            <v>그랜드스타렉스</v>
-          </cell>
-        </row>
-        <row r="37">
-          <cell r="A37">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="38">
-          <cell r="A38">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="39">
-          <cell r="A39">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="40">
-          <cell r="A40">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="41">
-          <cell r="A41">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="42">
-          <cell r="A42">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="43">
-          <cell r="A43">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="44">
-          <cell r="A44">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="45">
-          <cell r="A45">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="46">
-          <cell r="A46">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="47">
-          <cell r="A47">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="48">
-          <cell r="A48">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="49">
-          <cell r="A49">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="50">
-          <cell r="A50" t="str">
-            <v>포터초장축더블캡</v>
-          </cell>
-        </row>
-        <row r="51">
-          <cell r="A51" t="str">
-            <v>포터초장축슈퍼캡</v>
-          </cell>
-        </row>
-        <row r="52">
-          <cell r="A52">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="53">
-          <cell r="A53" t="str">
-            <v>포터</v>
-          </cell>
-        </row>
-        <row r="54">
-          <cell r="A54" t="str">
-            <v>포터장축켑</v>
-          </cell>
-        </row>
-        <row r="55">
-          <cell r="A55" t="str">
-            <v>포터초장축</v>
-          </cell>
-        </row>
-        <row r="56">
-          <cell r="A56" t="str">
-            <v>포터2</v>
-          </cell>
-        </row>
-        <row r="57">
-          <cell r="A57">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="58">
-          <cell r="A58" t="str">
-            <v>포터2내장탑</v>
-          </cell>
-        </row>
-        <row r="59">
-          <cell r="A59" t="str">
-            <v>포터2냉동탑</v>
-          </cell>
-        </row>
-        <row r="60">
-          <cell r="A60">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="61">
-          <cell r="A61">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="62">
-          <cell r="A62">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="63">
-          <cell r="A63">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="64">
-          <cell r="A64" t="str">
-            <v>현대5톤트럭</v>
-          </cell>
-        </row>
-        <row r="65">
-          <cell r="A65">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="66">
-          <cell r="A66">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="67">
-          <cell r="A67" t="str">
-            <v>스타렉스</v>
-          </cell>
-        </row>
-        <row r="68">
-          <cell r="A68" t="str">
-            <v>스타렉스인터쿨러9</v>
-          </cell>
-        </row>
-        <row r="69">
-          <cell r="A69" t="str">
-            <v>스타렉스9</v>
-          </cell>
-        </row>
-        <row r="70">
-          <cell r="A70">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="71">
-          <cell r="A71" t="str">
-            <v>스타렉스12</v>
-          </cell>
-        </row>
-        <row r="72">
-          <cell r="A72">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="73">
-          <cell r="A73" t="str">
-            <v>스타렉스6</v>
-          </cell>
-        </row>
-        <row r="74">
-          <cell r="A74">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="75">
-          <cell r="A75" t="str">
-            <v>스타렉스터보롱12</v>
-          </cell>
-        </row>
-        <row r="76">
-          <cell r="A76" t="str">
-            <v>스타렉스4륜</v>
-          </cell>
-        </row>
-        <row r="77">
-          <cell r="A77">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="78">
-          <cell r="A78" t="str">
-            <v>테라칸</v>
-          </cell>
-        </row>
-        <row r="79">
-          <cell r="A79">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="80">
-          <cell r="A80" t="str">
-            <v>베르나</v>
-          </cell>
-        </row>
-        <row r="81">
-          <cell r="A81" t="str">
-            <v>뉴베르나</v>
-          </cell>
-        </row>
-        <row r="82">
-          <cell r="A82" t="str">
-            <v>베르나하이브리드</v>
-          </cell>
-        </row>
-        <row r="83">
-          <cell r="A83">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="84">
-          <cell r="A84" t="str">
-            <v>카운티</v>
-          </cell>
-        </row>
-        <row r="85">
-          <cell r="A85" t="str">
-            <v>이-카운티</v>
-          </cell>
-        </row>
-        <row r="86">
-          <cell r="A86" t="str">
-            <v>벨로스터</v>
-          </cell>
-        </row>
-        <row r="87">
-          <cell r="A87" t="str">
-            <v>베르나</v>
-          </cell>
-        </row>
-        <row r="88">
-          <cell r="A88" t="str">
-            <v>아토스</v>
-          </cell>
-        </row>
-        <row r="89">
-          <cell r="A89" t="str">
-            <v>라비타</v>
-          </cell>
-        </row>
-        <row r="90">
-          <cell r="A90">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="91">
-          <cell r="A91" t="str">
-            <v>투싼</v>
-          </cell>
-        </row>
-        <row r="92">
-          <cell r="A92" t="str">
-            <v>투스카니</v>
-          </cell>
-        </row>
-        <row r="93">
-          <cell r="A93" t="str">
-            <v>티뷰론터뷸런스</v>
-          </cell>
-        </row>
-        <row r="94">
-          <cell r="A94">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="95">
-          <cell r="A95" t="str">
-            <v>쏘나타</v>
-          </cell>
-        </row>
-        <row r="96">
-          <cell r="A96" t="str">
-            <v>ef쏘나타</v>
-          </cell>
-        </row>
-        <row r="97">
-          <cell r="A97">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="98">
-          <cell r="A98" t="str">
-            <v>뉴EF쏘나타</v>
-          </cell>
-        </row>
-        <row r="99">
-          <cell r="A99" t="str">
-            <v>뉴EF쏘나타골드</v>
-          </cell>
-        </row>
-        <row r="100">
-          <cell r="A100" t="str">
-            <v>쏘나타 하이브리드</v>
-          </cell>
-        </row>
-        <row r="101">
-          <cell r="A101">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="102">
-          <cell r="A102" t="str">
-            <v>에쿠스</v>
-          </cell>
-        </row>
-        <row r="103">
-          <cell r="A103" t="str">
-            <v>i30</v>
-          </cell>
-        </row>
-        <row r="104">
-          <cell r="A104">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="105">
-          <cell r="A105" t="str">
-            <v>싼타페</v>
-          </cell>
-        </row>
-        <row r="106">
-          <cell r="A106" t="str">
-            <v>그랜저</v>
-          </cell>
-        </row>
-        <row r="107">
-          <cell r="A107" t="str">
-            <v>그랜저XG</v>
-          </cell>
-        </row>
-        <row r="108">
-          <cell r="A108" t="str">
-            <v>뉴그랜저XG</v>
-          </cell>
-        </row>
-        <row r="109">
-          <cell r="A109" t="str">
-            <v>그랜저TG</v>
-          </cell>
-        </row>
-        <row r="110">
-          <cell r="A110" t="str">
-            <v>로체</v>
-          </cell>
-        </row>
-        <row r="111">
-          <cell r="A111" t="str">
-            <v>포르테</v>
-          </cell>
-        </row>
-        <row r="112">
-          <cell r="A112" t="str">
-            <v>포르테쿱</v>
-          </cell>
-        </row>
-        <row r="113">
-          <cell r="A113" t="str">
-            <v>봉고</v>
-          </cell>
-        </row>
-        <row r="114">
-          <cell r="A114">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="115">
-          <cell r="A115" t="str">
-            <v>델타</v>
-          </cell>
-        </row>
-        <row r="116">
-          <cell r="A116" t="str">
-            <v>아벨라</v>
-          </cell>
-        </row>
-        <row r="117">
-          <cell r="A117" t="str">
-            <v>쎄라토</v>
-          </cell>
-        </row>
-        <row r="118">
-          <cell r="A118" t="str">
-            <v>k5</v>
-          </cell>
-        </row>
-        <row r="119">
-          <cell r="A119" t="str">
-            <v>k5 하이브리드</v>
-          </cell>
-        </row>
-        <row r="120">
-          <cell r="A120" t="str">
-            <v>리오</v>
-          </cell>
-        </row>
-        <row r="121">
-          <cell r="A121" t="str">
-            <v>리오RX-V</v>
-          </cell>
-        </row>
-        <row r="122">
-          <cell r="A122" t="str">
-            <v>리오sf</v>
-          </cell>
-        </row>
-        <row r="123">
-          <cell r="A123" t="str">
-            <v>세피아</v>
-          </cell>
-        </row>
-        <row r="124">
-          <cell r="A124" t="str">
-            <v>세피아2</v>
-          </cell>
-        </row>
-        <row r="125">
-          <cell r="A125" t="str">
-            <v>세피아오토</v>
-          </cell>
-        </row>
-        <row r="126">
-          <cell r="A126" t="str">
-            <v>스펙트라</v>
-          </cell>
-        </row>
-        <row r="127">
-          <cell r="A127" t="str">
-            <v>스펙트라윙</v>
-          </cell>
-        </row>
-        <row r="128">
-          <cell r="A128" t="str">
-            <v>비스토</v>
-          </cell>
-        </row>
-        <row r="129">
-          <cell r="A129" t="str">
-            <v>슈마</v>
-          </cell>
-        </row>
-        <row r="130">
-          <cell r="A130" t="str">
-            <v>프라이드웨곤</v>
-          </cell>
-        </row>
-        <row r="131">
-          <cell r="A131" t="str">
-            <v>프라이드</v>
-          </cell>
-        </row>
-        <row r="132">
-          <cell r="A132">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="133">
-          <cell r="A133" t="str">
-            <v>프런티어</v>
-          </cell>
-        </row>
-        <row r="134">
-          <cell r="A134">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="135">
-          <cell r="A135" t="str">
-            <v>스포티지</v>
-          </cell>
-        </row>
-        <row r="137">
-          <cell r="A137" t="str">
-            <v>프런티어1.3톤</v>
-          </cell>
-        </row>
-        <row r="138">
-          <cell r="A138" t="str">
-            <v>오텍봉고킹캡</v>
-          </cell>
-        </row>
-        <row r="139">
-          <cell r="A139">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="140">
-          <cell r="A140" t="str">
-            <v>프런티어1.4톤</v>
-          </cell>
-        </row>
-        <row r="141">
-          <cell r="A141" t="str">
-            <v>봉고킹캡</v>
-          </cell>
-        </row>
-        <row r="142">
-          <cell r="A142">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="143">
-          <cell r="A143" t="str">
-            <v>오텍프런티어</v>
-          </cell>
-        </row>
-        <row r="144">
-          <cell r="A144">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="145">
-          <cell r="A145" t="str">
-            <v>봉고3</v>
-          </cell>
-        </row>
-        <row r="146">
-          <cell r="A146" t="str">
-            <v>봉고3 1.2</v>
-          </cell>
-        </row>
-        <row r="147">
-          <cell r="A147" t="str">
-            <v>봉고3 1.4</v>
-          </cell>
-        </row>
-        <row r="148">
-          <cell r="A148" t="str">
-            <v>봉고3 1톤</v>
-          </cell>
-        </row>
-        <row r="149">
-          <cell r="A149" t="str">
-            <v>봉고3 카고</v>
-          </cell>
-        </row>
-        <row r="150">
-          <cell r="A150" t="str">
-            <v>봉고3 플러스</v>
-          </cell>
-        </row>
-        <row r="151">
-          <cell r="A151" t="str">
-            <v>봉고프런티어킹캡</v>
-          </cell>
-        </row>
-        <row r="152">
-          <cell r="A152" t="str">
-            <v>봉고프런티어4륜</v>
-          </cell>
-        </row>
-        <row r="153">
-          <cell r="A153" t="str">
-            <v>봉고프런티어</v>
-          </cell>
-        </row>
-        <row r="154">
-          <cell r="A154" t="str">
-            <v>봉고3 탑</v>
-          </cell>
-        </row>
-        <row r="155">
-          <cell r="A155" t="str">
-            <v>봉고 트런티어 탑</v>
-          </cell>
-        </row>
-        <row r="156">
-          <cell r="A156" t="str">
-            <v>봉고프런티어 GLS</v>
-          </cell>
-        </row>
-        <row r="157">
-          <cell r="A157" t="str">
-            <v>마티즈</v>
-          </cell>
-        </row>
-        <row r="158">
-          <cell r="A158" t="str">
-            <v>마티즈0.8at</v>
-          </cell>
-        </row>
-        <row r="159">
-          <cell r="A159" t="str">
-            <v>마티즈0.8mt</v>
-          </cell>
-        </row>
-        <row r="160">
-          <cell r="A160" t="str">
-            <v>마티즈밴 AT</v>
-          </cell>
-        </row>
-        <row r="161">
-          <cell r="A161">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="162">
-          <cell r="A162" t="str">
-            <v>윈스톰</v>
-          </cell>
-        </row>
-        <row r="163">
-          <cell r="A163" t="str">
-            <v>라노스1.3</v>
-          </cell>
-        </row>
-        <row r="164">
-          <cell r="A164" t="str">
-            <v>라노스1.5</v>
-          </cell>
-        </row>
-        <row r="165">
-          <cell r="A165" t="str">
-            <v>라노스해치백1.3</v>
-          </cell>
-        </row>
-        <row r="166">
-          <cell r="A166" t="str">
-            <v>라노스해치백1.5</v>
-          </cell>
-        </row>
-        <row r="167">
-          <cell r="A167" t="str">
-            <v>라노스</v>
-          </cell>
-        </row>
-        <row r="168">
-          <cell r="A168">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="169">
-          <cell r="A169" t="str">
-            <v>매그너스</v>
-          </cell>
-        </row>
-        <row r="170">
-          <cell r="A170">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="171">
-          <cell r="A171" t="str">
-            <v>누비라1.5</v>
-          </cell>
-        </row>
-        <row r="173">
-          <cell r="A173" t="str">
-            <v>라세티1.6</v>
-          </cell>
-        </row>
-        <row r="174">
-          <cell r="A174">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="175">
-          <cell r="A175">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="176">
-          <cell r="A176" t="str">
-            <v>라세티5</v>
-          </cell>
-        </row>
-        <row r="177">
-          <cell r="A177" t="str">
-            <v>라세티5 mt</v>
-          </cell>
-        </row>
-        <row r="178">
-          <cell r="A178">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="179">
-          <cell r="A179" t="str">
-            <v>라세티1.5</v>
-          </cell>
-        </row>
-        <row r="180">
-          <cell r="A180">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="181">
-          <cell r="A181" t="str">
-            <v>젠트라1.5</v>
-          </cell>
-        </row>
-        <row r="182">
-          <cell r="A182" t="str">
-            <v>젠트라1.6</v>
-          </cell>
-        </row>
-        <row r="183">
-          <cell r="A183" t="str">
-            <v>젠트라1.2</v>
-          </cell>
-        </row>
-        <row r="185">
-          <cell r="A185" t="str">
-            <v>칼로스1.2</v>
-          </cell>
-        </row>
-        <row r="186">
-          <cell r="A186" t="str">
-            <v>칼로스1.5</v>
-          </cell>
-        </row>
-        <row r="187">
-          <cell r="A187" t="str">
-            <v>티코</v>
-          </cell>
-        </row>
-        <row r="188">
-          <cell r="A188" t="str">
-            <v>다마스</v>
-          </cell>
-        </row>
-        <row r="189">
-          <cell r="A189" t="str">
-            <v>다마스밴</v>
-          </cell>
-        </row>
-        <row r="190">
-          <cell r="A190" t="str">
-            <v>다마스5</v>
-          </cell>
-        </row>
-        <row r="191">
-          <cell r="A191" t="str">
-            <v>다마스7</v>
-          </cell>
-        </row>
-        <row r="192">
-          <cell r="A192" t="str">
-            <v>레간자</v>
-          </cell>
-        </row>
-        <row r="193">
-          <cell r="A193" t="str">
-            <v>레간자2.0</v>
-          </cell>
-        </row>
-        <row r="194">
-          <cell r="A194" t="str">
-            <v>라보</v>
-          </cell>
-        </row>
-        <row r="195">
-          <cell r="A195" t="str">
-            <v>라보롱카고</v>
-          </cell>
-        </row>
-        <row r="196">
-          <cell r="A196">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="197">
-          <cell r="A197" t="str">
-            <v>라보5MT</v>
-          </cell>
-        </row>
-        <row r="198">
-          <cell r="A198" t="str">
-            <v>CR-V</v>
-          </cell>
-        </row>
-        <row r="199">
-          <cell r="A199" t="str">
-            <v>쏘울</v>
-          </cell>
-        </row>
-        <row r="200">
-          <cell r="A200" t="str">
-            <v>모닝</v>
-          </cell>
-        </row>
-        <row r="201">
-          <cell r="A201" t="str">
-            <v>쏘렌토</v>
-          </cell>
-        </row>
-        <row r="202">
-          <cell r="A202" t="str">
-            <v>쏘렌토gl</v>
-          </cell>
-        </row>
-        <row r="203">
-          <cell r="A203" t="str">
-            <v>쏘렌토GLS</v>
-          </cell>
-        </row>
-        <row r="204">
-          <cell r="A204">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="205">
-          <cell r="A205" t="str">
-            <v>파맥스</v>
-          </cell>
-        </row>
-        <row r="206">
-          <cell r="A206" t="str">
-            <v>타우너</v>
-          </cell>
-        </row>
-        <row r="207">
-          <cell r="A207" t="str">
-            <v>프레지오</v>
-          </cell>
-        </row>
-        <row r="208">
-          <cell r="A208">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="209">
-          <cell r="A209">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="210">
-          <cell r="A210">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="211">
-          <cell r="A211">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="212">
-          <cell r="A212" t="str">
-            <v>오피러스</v>
-          </cell>
-        </row>
-        <row r="213">
-          <cell r="A213" t="str">
-            <v>옵티마</v>
-          </cell>
-        </row>
-        <row r="214">
-          <cell r="A214" t="str">
-            <v>옵티마리갈</v>
-          </cell>
-        </row>
-        <row r="215">
-          <cell r="A215" t="str">
-            <v>sm3</v>
-          </cell>
-        </row>
-        <row r="216">
-          <cell r="A216">
-            <v>520</v>
-          </cell>
-        </row>
-        <row r="217">
-          <cell r="A217" t="str">
-            <v>520 LPG</v>
-          </cell>
-        </row>
-        <row r="218">
-          <cell r="A218">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="219">
-          <cell r="A219" t="str">
-            <v>525V</v>
-          </cell>
-        </row>
-        <row r="220">
-          <cell r="A220" t="str">
-            <v>520v</v>
-          </cell>
-        </row>
-        <row r="221">
-          <cell r="A221">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="222">
-          <cell r="A222" t="str">
-            <v>시에로</v>
-          </cell>
-        </row>
-        <row r="223">
-          <cell r="A223">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="224">
-          <cell r="A224">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="225">
-          <cell r="A225">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="226">
-          <cell r="A226">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="227">
-          <cell r="A227">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="228">
-          <cell r="A228">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="229">
-          <cell r="A229" t="str">
-            <v>bmw525i</v>
-          </cell>
-        </row>
-        <row r="230">
-          <cell r="A230">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="231">
-          <cell r="A231">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="232">
-          <cell r="A232">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="233">
-          <cell r="A233">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="234">
-          <cell r="A234">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="235">
-          <cell r="A235" t="str">
-            <v>무쏘</v>
-          </cell>
-        </row>
-        <row r="236">
-          <cell r="A236" t="str">
-            <v>뉴무쏘</v>
-          </cell>
-        </row>
-        <row r="237">
-          <cell r="A237" t="str">
-            <v>카니발</v>
-          </cell>
-        </row>
-        <row r="238">
-          <cell r="A238" t="str">
-            <v>카니발2</v>
-          </cell>
-        </row>
-        <row r="239">
-          <cell r="A239" t="str">
-            <v>카렌스</v>
-          </cell>
-        </row>
-        <row r="240">
-          <cell r="A240" t="str">
-            <v>렉스턴</v>
-          </cell>
-        </row>
-        <row r="241">
-          <cell r="A241" t="str">
-            <v>체어맨</v>
-          </cell>
-        </row>
-        <row r="242">
-          <cell r="A242">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="243">
-          <cell r="A243">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="244">
-          <cell r="A244" t="str">
-            <v>이스타나</v>
-          </cell>
-        </row>
-        <row r="245">
-          <cell r="A245" t="str">
-            <v>이스타나15</v>
-          </cell>
-        </row>
-        <row r="246">
-          <cell r="A246" t="str">
-            <v>이스타나12</v>
-          </cell>
-        </row>
-        <row r="247">
-          <cell r="A247" t="str">
-            <v>이스타나6밴</v>
-          </cell>
-        </row>
-        <row r="248">
-          <cell r="A248" t="str">
-            <v>엑티언</v>
-          </cell>
-        </row>
-        <row r="249">
-          <cell r="A249" t="str">
-            <v>엑티언스포츠</v>
-          </cell>
-        </row>
-        <row r="250">
-          <cell r="A250" t="str">
-            <v>코란도</v>
-          </cell>
-        </row>
-        <row r="251">
-          <cell r="A251" t="str">
-            <v>렉서스ES330</v>
-          </cell>
-        </row>
-        <row r="252">
-          <cell r="A252" t="str">
-            <v>렉서스ES350</v>
-          </cell>
-        </row>
-        <row r="253">
-          <cell r="A253" t="str">
-            <v>렉서스LS430</v>
-          </cell>
-        </row>
-        <row r="254">
-          <cell r="A254" t="str">
-            <v>렉서스GS300</v>
-          </cell>
-        </row>
-        <row r="255">
-          <cell r="A255" t="str">
-            <v>렉서스LS460</v>
-          </cell>
-        </row>
-        <row r="256">
-          <cell r="A256" t="str">
-            <v>렉서스LS460L</v>
-          </cell>
-        </row>
-        <row r="257">
-          <cell r="A257" t="str">
-            <v>벤츠 C-240</v>
-          </cell>
-        </row>
-        <row r="258">
-          <cell r="A258" t="str">
-            <v>아우디a6</v>
-          </cell>
-        </row>
-        <row r="259">
-          <cell r="A259" t="str">
-            <v>아우디a4</v>
-          </cell>
-        </row>
-        <row r="260">
-          <cell r="A260" t="str">
-            <v>엑센트</v>
-          </cell>
-        </row>
-        <row r="261">
-          <cell r="A261" t="str">
-            <v>스타렉스인터쿨러9인4WD</v>
-          </cell>
-        </row>
-        <row r="262">
-          <cell r="A262" t="str">
-            <v>스타렉스9</v>
-          </cell>
-        </row>
-        <row r="263">
-          <cell r="A263" t="str">
-            <v>뉴스타렉스4륜AT</v>
-          </cell>
-        </row>
-        <row r="264">
-          <cell r="A264" t="str">
-            <v>스타렉스인터쿨러단축9인</v>
-          </cell>
-        </row>
-        <row r="265">
-          <cell r="A265" t="str">
-            <v>프라이드해치백</v>
-          </cell>
-        </row>
-        <row r="266">
-          <cell r="A266" t="str">
-            <v>싼타페AT</v>
-          </cell>
-        </row>
-        <row r="267">
-          <cell r="A267" t="str">
-            <v>뉴스타렉스12</v>
-          </cell>
-        </row>
-        <row r="268">
-          <cell r="A268" t="str">
-            <v>포터II냉동탑차</v>
-          </cell>
-        </row>
-        <row r="269">
-          <cell r="A269" t="str">
-            <v>포터II슈퍼캡냉동탑차</v>
-          </cell>
-        </row>
-        <row r="270">
-          <cell r="A270" t="str">
-            <v>다마스5인승</v>
-          </cell>
-        </row>
-        <row r="271">
-          <cell r="A271" t="str">
-            <v>카운티25</v>
-          </cell>
-        </row>
-        <row r="272">
-          <cell r="A272" t="str">
-            <v>프라이드가솔린해치</v>
-          </cell>
-        </row>
-        <row r="273">
-          <cell r="A273" t="str">
-            <v>봉고 III 코치15</v>
-          </cell>
-        </row>
-        <row r="274">
-          <cell r="A274" t="str">
-            <v>그레이스15인승</v>
-          </cell>
-        </row>
-        <row r="275">
-          <cell r="A275" t="str">
-            <v>프라이드해치백디젤</v>
-          </cell>
-        </row>
-        <row r="276">
-          <cell r="A276" t="str">
-            <v>올뉴마티즈</v>
-          </cell>
-        </row>
-        <row r="277">
-          <cell r="A277" t="str">
-            <v>갤로퍼</v>
-          </cell>
-        </row>
-        <row r="278">
-          <cell r="A278" t="str">
-            <v>그랜드스타렉스12</v>
-          </cell>
-        </row>
-        <row r="279">
-          <cell r="A279" t="str">
-            <v>투싼 AT</v>
-          </cell>
-        </row>
-        <row r="280">
-          <cell r="A280" t="str">
-            <v>봉고 III 1.2톤카고</v>
-          </cell>
-        </row>
-        <row r="281">
-          <cell r="A281" t="str">
-            <v>투싼 CRDI</v>
-          </cell>
-        </row>
-        <row r="282">
-          <cell r="A282" t="str">
-            <v>카운티25</v>
-          </cell>
-        </row>
-        <row r="283">
-          <cell r="A283" t="str">
-            <v>그레이스터보15인</v>
-          </cell>
-        </row>
-        <row r="284">
-          <cell r="A284" t="str">
-            <v>그레이스터보15인승</v>
-          </cell>
-        </row>
-        <row r="285">
-          <cell r="A285" t="str">
-            <v>포터II냉동탑차</v>
-          </cell>
-        </row>
-        <row r="286">
-          <cell r="A286" t="str">
-            <v>봉고 III 코치15</v>
-          </cell>
-        </row>
-        <row r="287">
-          <cell r="A287" t="str">
-            <v>봉고 III 1톤카고</v>
-          </cell>
-        </row>
-        <row r="288">
-          <cell r="A288" t="str">
-            <v>봉고III 코치</v>
-          </cell>
-        </row>
-        <row r="289">
-          <cell r="A289" t="str">
-            <v>봉고III 1톤</v>
-          </cell>
-        </row>
-        <row r="290">
-          <cell r="A290" t="str">
-            <v>봉고 III 12인승</v>
-          </cell>
-        </row>
-        <row r="291">
-          <cell r="A291" t="str">
-            <v>오텍파라메딕특수구급차</v>
-          </cell>
-        </row>
-        <row r="292">
-          <cell r="A292" t="str">
-            <v>봉고 III 카고</v>
-          </cell>
-        </row>
-        <row r="293">
-          <cell r="A293" t="str">
-            <v>스타렉스4wdAT</v>
-          </cell>
-        </row>
-        <row r="294">
-          <cell r="A294" t="str">
-            <v>포터II 카고</v>
-          </cell>
-        </row>
-        <row r="295">
-          <cell r="A295" t="str">
-            <v>프라이드1.6</v>
-          </cell>
-        </row>
-        <row r="296">
-          <cell r="A296" t="str">
-            <v>스타렉스7인승</v>
-          </cell>
-        </row>
-        <row r="297">
-          <cell r="A297" t="str">
-            <v>뉴스타렉스9</v>
-          </cell>
-        </row>
-        <row r="298">
-          <cell r="A298" t="str">
-            <v>봉고III냉탑</v>
-          </cell>
-        </row>
-        <row r="299">
-          <cell r="A299" t="str">
-            <v>프라이드해치백디젤</v>
-          </cell>
-        </row>
-        <row r="300">
-          <cell r="A300" t="str">
-            <v>테라칸ex</v>
-          </cell>
-        </row>
-        <row r="301">
-          <cell r="A301" t="str">
-            <v>라세티</v>
-          </cell>
-        </row>
-        <row r="302">
-          <cell r="A302" t="str">
-            <v>뉴스타렉스12</v>
-          </cell>
-        </row>
-        <row r="303">
-          <cell r="A303" t="str">
-            <v>봉고III코치</v>
-          </cell>
-        </row>
-        <row r="304">
-          <cell r="A304" t="str">
-            <v>뉴스타렉스</v>
-          </cell>
-        </row>
-        <row r="305">
-          <cell r="A305" t="str">
-            <v>테라칸 JX250</v>
-          </cell>
-        </row>
-        <row r="306">
-          <cell r="A306" t="str">
-            <v>스타렉스4륜</v>
-          </cell>
-        </row>
-        <row r="307">
-          <cell r="A307" t="str">
-            <v>뉴스타렉스사륜</v>
-          </cell>
-        </row>
-        <row r="308">
-          <cell r="A308" t="str">
-            <v>라세티해치백가솔린</v>
-          </cell>
-        </row>
-        <row r="309">
-          <cell r="A309" t="str">
-            <v>스타렉스사륜</v>
-          </cell>
-        </row>
-        <row r="310">
-          <cell r="A310" t="str">
-            <v>갤로퍼II승합</v>
-          </cell>
-        </row>
-        <row r="311">
-          <cell r="A311" t="str">
-            <v>갤로퍼</v>
-          </cell>
-        </row>
-        <row r="312">
-          <cell r="A312" t="str">
-            <v>라세티해치백</v>
-          </cell>
-        </row>
-        <row r="313">
-          <cell r="A313" t="str">
-            <v>뉴스타렉스12인승2륜</v>
-          </cell>
-        </row>
-        <row r="314">
-          <cell r="A314">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="315">
-          <cell r="A315">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="316">
-          <cell r="A316">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="317">
-          <cell r="A317">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="318">
-          <cell r="A318">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="319">
-          <cell r="A319">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="320">
-          <cell r="A320">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="321">
-          <cell r="A321">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="322">
-          <cell r="A322">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="323">
-          <cell r="A323">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="324">
-          <cell r="A324">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="325">
-          <cell r="A325">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="326">
-          <cell r="A326">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="327">
-          <cell r="A327">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="328">
-          <cell r="A328">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="329">
-          <cell r="A329">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="330">
-          <cell r="A330">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="331">
-          <cell r="A331">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="332">
-          <cell r="A332">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="333">
-          <cell r="A333">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="334">
-          <cell r="A334">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="335">
-          <cell r="A335">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="336">
-          <cell r="A336">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="337">
-          <cell r="A337">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="338">
-          <cell r="A338">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="339">
-          <cell r="A339">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="340">
-          <cell r="A340">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="341">
-          <cell r="A341">
-            <v>518</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6">
-        <row r="2">
-          <cell r="G2" t="str">
-            <v>KJ1705-22</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="B3">
-            <v>2017</v>
-          </cell>
-          <cell r="C3">
-            <v>5</v>
-          </cell>
-          <cell r="G3">
-            <v>5</v>
-          </cell>
-          <cell r="J3">
-            <v>42856</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="J4">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="B12">
-            <v>5</v>
-          </cell>
-          <cell r="C12">
-            <v>5</v>
-          </cell>
-          <cell r="D12">
-            <v>5</v>
-          </cell>
-          <cell r="E12">
-            <v>5</v>
-          </cell>
-          <cell r="F12">
-            <v>5</v>
-          </cell>
-          <cell r="G12">
-            <v>5</v>
-          </cell>
-          <cell r="H12">
-            <v>5</v>
-          </cell>
-          <cell r="I12">
-            <v>5</v>
-          </cell>
-          <cell r="J12">
-            <v>5</v>
-          </cell>
-          <cell r="K12">
-            <v>0</v>
-          </cell>
-          <cell r="L12">
-            <v>0</v>
-          </cell>
-          <cell r="M12">
-            <v>0</v>
-          </cell>
-          <cell r="N12">
-            <v>0</v>
-          </cell>
-          <cell r="Q12">
-            <v>0</v>
-          </cell>
-          <cell r="R12">
-            <v>0</v>
-          </cell>
-          <cell r="S12">
-            <v>0</v>
-          </cell>
-          <cell r="T12">
-            <v>31</v>
-          </cell>
-          <cell r="U12">
-            <v>0</v>
-          </cell>
-          <cell r="V12">
-            <v>0</v>
-          </cell>
-          <cell r="X12">
-            <v>0</v>
-          </cell>
-          <cell r="Y12">
-            <v>0</v>
-          </cell>
-          <cell r="Z12">
-            <v>0</v>
-          </cell>
-          <cell r="AB12">
-            <v>0</v>
-          </cell>
-          <cell r="AC12">
-            <v>0</v>
-          </cell>
-          <cell r="AD12">
-            <v>0</v>
-          </cell>
-          <cell r="AE12">
-            <v>0</v>
-          </cell>
-          <cell r="AF12">
-            <v>0</v>
-          </cell>
-          <cell r="AG12">
-            <v>0</v>
-          </cell>
-          <cell r="AH12">
-            <v>0</v>
-          </cell>
-          <cell r="AI12">
-            <v>0</v>
-          </cell>
-          <cell r="AJ12">
-            <v>0</v>
-          </cell>
-          <cell r="AK12">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="B13">
-            <v>0</v>
-          </cell>
-          <cell r="C13">
-            <v>0</v>
-          </cell>
-          <cell r="D13" t="str">
-            <v>매매계약서</v>
-          </cell>
-          <cell r="E13">
-            <v>0</v>
-          </cell>
-          <cell r="F13">
-            <v>0</v>
-          </cell>
-          <cell r="G13">
-            <v>0</v>
-          </cell>
-          <cell r="H13" t="str">
-            <v>재고</v>
-          </cell>
-          <cell r="I13">
-            <v>284</v>
-          </cell>
-          <cell r="J13">
-            <v>284</v>
-          </cell>
-          <cell r="K13">
-            <v>284</v>
-          </cell>
-          <cell r="L13">
-            <v>31</v>
-          </cell>
-          <cell r="M13">
-            <v>31</v>
-          </cell>
-          <cell r="N13">
-            <v>31</v>
-          </cell>
-          <cell r="Q13">
-            <v>31</v>
-          </cell>
-          <cell r="R13">
-            <v>31</v>
-          </cell>
-          <cell r="S13">
-            <v>31</v>
-          </cell>
-          <cell r="T13">
-            <v>31</v>
-          </cell>
-          <cell r="U13">
-            <v>31</v>
-          </cell>
-          <cell r="V13">
-            <v>31</v>
-          </cell>
-          <cell r="W13">
-            <v>31</v>
-          </cell>
-          <cell r="X13">
-            <v>31</v>
-          </cell>
-          <cell r="Y13">
-            <v>31</v>
-          </cell>
-          <cell r="Z13">
-            <v>31</v>
-          </cell>
-          <cell r="AB13">
-            <v>31</v>
-          </cell>
-          <cell r="AC13">
-            <v>31</v>
-          </cell>
-          <cell r="AD13">
-            <v>31</v>
-          </cell>
-          <cell r="AE13">
-            <v>31</v>
-          </cell>
-          <cell r="AF13">
-            <v>31</v>
-          </cell>
-          <cell r="AG13">
-            <v>31</v>
-          </cell>
-          <cell r="AH13">
-            <v>31</v>
-          </cell>
-          <cell r="AI13">
-            <v>31</v>
-          </cell>
-          <cell r="AJ13">
-            <v>31</v>
-          </cell>
-          <cell r="AK13">
-            <v>31</v>
-          </cell>
-          <cell r="AL13" t="str">
-            <v>전체</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="B14" t="str">
-            <v>구분입력</v>
-          </cell>
-          <cell r="C14" t="str">
-            <v>2회사</v>
-          </cell>
-          <cell r="D14" t="str">
-            <v>3번호</v>
-          </cell>
-          <cell r="E14" t="str">
-            <v>4날짜</v>
-          </cell>
-          <cell r="F14" t="str">
-            <v>5차번</v>
-          </cell>
-          <cell r="G14" t="str">
-            <v>6차명</v>
-          </cell>
-          <cell r="H14" t="str">
-            <v>7연식</v>
-          </cell>
-          <cell r="I14" t="str">
-            <v>8세금계산서</v>
-          </cell>
-          <cell r="J14" t="str">
-            <v>9면장액</v>
-          </cell>
-          <cell r="K14" t="str">
-            <v>10영세율</v>
-          </cell>
-          <cell r="L14" t="str">
-            <v>11등록번호</v>
-          </cell>
-          <cell r="M14" t="str">
-            <v>12매출일</v>
-          </cell>
-          <cell r="N14" t="str">
-            <v>13차대번호</v>
-          </cell>
-          <cell r="O14" t="str">
-            <v>14말소일</v>
-          </cell>
-          <cell r="P14" t="str">
-            <v>15관청</v>
-          </cell>
-          <cell r="Q14" t="str">
-            <v>16메모</v>
-          </cell>
-          <cell r="R14" t="str">
-            <v>17면장</v>
-          </cell>
-          <cell r="S14" t="str">
-            <v>18면장번호</v>
-          </cell>
-          <cell r="T14" t="str">
-            <v>선적
-업체20</v>
-          </cell>
-          <cell r="U14" t="str">
-            <v>b/l no.21</v>
-          </cell>
-          <cell r="V14" t="str">
-            <v>21색깔</v>
-          </cell>
-          <cell r="W14" t="str">
-            <v>도착지22</v>
-          </cell>
-          <cell r="X14" t="str">
-            <v>매입처23</v>
-          </cell>
-          <cell r="Y14" t="str">
-            <v>CONSIGNEE24</v>
-          </cell>
-          <cell r="Z14" t="str">
-            <v>팩스25</v>
-          </cell>
-          <cell r="AA14" t="str">
-            <v>전화번호26</v>
-          </cell>
-          <cell r="AB14" t="str">
-            <v>실매입금27</v>
-          </cell>
-          <cell r="AC14" t="str">
-            <v>선입금28</v>
-          </cell>
-          <cell r="AD14" t="str">
-            <v>잔금29</v>
-          </cell>
-          <cell r="AE14" t="str">
-            <v>실거래 차액30</v>
-          </cell>
-          <cell r="AF14" t="str">
-            <v>차액받은날</v>
-          </cell>
-          <cell r="AG14" t="str">
-            <v>수출이행32</v>
-          </cell>
-          <cell r="AH14" t="str">
-            <v>계산서/환급33</v>
-          </cell>
-          <cell r="AI14" t="str">
-            <v>차주성명34</v>
-          </cell>
-          <cell r="AJ14" t="str">
-            <v>주민등록번호35</v>
-          </cell>
-          <cell r="AK14" t="str">
-            <v>주소36</v>
-          </cell>
-          <cell r="AL14" t="str">
-            <v>현재고</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="B15">
-            <v>530</v>
-          </cell>
-          <cell r="C15" t="str">
-            <v>성신</v>
-          </cell>
-          <cell r="D15" t="str">
-            <v>1 / No.1</v>
-          </cell>
-          <cell r="E15">
-            <v>42873.019456018519</v>
-          </cell>
-          <cell r="F15" t="str">
-            <v>마티즈</v>
-          </cell>
-          <cell r="G15" t="str">
-            <v xml:space="preserve">DAEWOO  MATIZ </v>
-          </cell>
-          <cell r="H15" t="str">
-            <v>2001</v>
-          </cell>
-          <cell r="I15">
-            <v>42873</v>
-          </cell>
-          <cell r="J15">
-            <v>0</v>
-          </cell>
-          <cell r="K15">
-            <v>1600000</v>
-          </cell>
-          <cell r="L15" t="str">
-            <v>17소8195</v>
-          </cell>
-          <cell r="M15">
-            <v>1600000</v>
-          </cell>
-          <cell r="N15" t="str">
-            <v>KLY4A11BD1C726117</v>
-          </cell>
-          <cell r="O15">
-            <v>42607</v>
-          </cell>
-          <cell r="P15" t="str">
-            <v>인천광역시 연수구청장</v>
-          </cell>
-          <cell r="Q15">
-            <v>42607</v>
-          </cell>
-          <cell r="R15">
-            <v>42768</v>
-          </cell>
-          <cell r="S15">
-            <v>4374</v>
-          </cell>
-          <cell r="T15">
-            <v>4374</v>
-          </cell>
-          <cell r="U15">
-            <v>4374</v>
-          </cell>
-          <cell r="V15">
-            <v>4374</v>
-          </cell>
-          <cell r="W15" t="str">
-            <v>UZB</v>
-          </cell>
-          <cell r="X15" t="str">
-            <v>구자견 이사</v>
-          </cell>
-          <cell r="Y15" t="str"/>
-          <cell r="Z15">
-            <v>0</v>
-          </cell>
-          <cell r="AA15">
-            <v>0</v>
-          </cell>
-          <cell r="AB15">
-            <v>0</v>
-          </cell>
-          <cell r="AC15">
-            <v>0</v>
-          </cell>
-          <cell r="AD15">
-            <v>0</v>
-          </cell>
-          <cell r="AE15">
-            <v>0</v>
-          </cell>
-          <cell r="AF15">
-            <v>0</v>
-          </cell>
-          <cell r="AG15">
-            <v>0</v>
-          </cell>
-          <cell r="AH15" t="str">
-            <v>개인</v>
-          </cell>
-          <cell r="AI15" t="str">
-            <v>김용식</v>
-          </cell>
-          <cell r="AJ15" t="str">
-            <v>650704-1471211</v>
-          </cell>
-          <cell r="AK15" t="str">
-            <v>인천시 부평구 장제로 28번길</v>
-          </cell>
-          <cell r="AL15" t="str">
-            <v>SSYA1701</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-      <sheetData sheetId="21"/>
-      <sheetData sheetId="22"/>
-      <sheetData sheetId="23"/>
-      <sheetData sheetId="24"/>
-      <sheetData sheetId="25"/>
-      <sheetData sheetId="26"/>
-      <sheetData sheetId="27" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink8.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="12 (3)"/>
-      <sheetName val="1"/>
-      <sheetName val="1(2)"/>
-      <sheetName val="2"/>
-      <sheetName val="2 (2)"/>
-      <sheetName val="3"/>
-      <sheetName val="3(2)"/>
-      <sheetName val="4"/>
-      <sheetName val="4 (2)"/>
-      <sheetName val="5"/>
-      <sheetName val="5 (2)"/>
-      <sheetName val="6"/>
-      <sheetName val="6 (2)"/>
-      <sheetName val="7"/>
-      <sheetName val="7 (2)"/>
-      <sheetName val="8"/>
-      <sheetName val="8 (2)"/>
-      <sheetName val="9"/>
-      <sheetName val="9 (2)"/>
-      <sheetName val="10"/>
-      <sheetName val="10 (2)"/>
-      <sheetName val="11"/>
-      <sheetName val="11 (2)"/>
-      <sheetName val="12"/>
-      <sheetName val="12 (2)"/>
-      <sheetName val="집계표"/>
-      <sheetName val="잔액"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13" refreshError="1"/>
-      <sheetData sheetId="14" refreshError="1"/>
-      <sheetData sheetId="15" refreshError="1"/>
-      <sheetData sheetId="16" refreshError="1"/>
-      <sheetData sheetId="17" refreshError="1"/>
-      <sheetData sheetId="18" refreshError="1"/>
-      <sheetData sheetId="19" refreshError="1"/>
-      <sheetData sheetId="20" refreshError="1"/>
-      <sheetData sheetId="21" refreshError="1"/>
-      <sheetData sheetId="22" refreshError="1"/>
-      <sheetData sheetId="23" refreshError="1"/>
-      <sheetData sheetId="24"/>
-      <sheetData sheetId="25" refreshError="1"/>
-      <sheetData sheetId="26" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink9.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="20161130이후"/>
-      <sheetName val="CarName_INPUT입력"/>
-      <sheetName val="쉬핑마크 (2)"/>
-      <sheetName val="쉬핑마크"/>
-      <sheetName val="계약서"/>
-      <sheetName val="쉬핑INVOICE"/>
-      <sheetName val="수출현황_종합"/>
-      <sheetName val="부품"/>
-      <sheetName val="차량매입경비신청서 (2)"/>
-      <sheetName val="신한 원화"/>
-      <sheetName val="코리아 원화"/>
-      <sheetName val="차량매입경비신청서"/>
-      <sheetName val="면장신청"/>
-      <sheetName val="Sheet2"/>
-      <sheetName val="Sheet3"/>
-      <sheetName val="말소신청서"/>
-      <sheetName val="월말신고"/>
-      <sheetName val="구매선적일보"/>
-      <sheetName val="매입현황 보고"/>
-      <sheetName val="재고관리"/>
-      <sheetName val="말소증"/>
-      <sheetName val="매매계약서"/>
-      <sheetName val="면장주소"/>
-      <sheetName val="현금영수증"/>
-      <sheetName val="이행신고서"/>
-      <sheetName val="개인정보"/>
-      <sheetName val="Sheet1"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>차명</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>엑센트1495</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>엑센트1396</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>엑센트1341</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8" t="str">
-            <v>엑센트1591</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9" t="str">
-            <v>엑센트1368</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10" t="str">
-            <v>엑센트1582</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11" t="str">
-            <v>엑센트</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12" t="str">
-            <v>아반떼</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13" t="str">
-            <v>md</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14" t="str">
-            <v>아반떼오토</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="A15" t="str">
-            <v>hd</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="A16" t="str">
-            <v>xd</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="A17" t="str">
-            <v>뉴아반떼</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="A18" t="str">
-            <v>클릭</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="A19" t="str">
-            <v>뉴클릭</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="A20" t="str">
-            <v>엘란트라</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="A21" t="str">
-            <v>그레이스</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="A22" t="str">
-            <v>그레이스9</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="A23" t="str">
-            <v>그레이스12</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="A24">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="A25" t="str">
-            <v>그레이스15</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="A26">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="A27" t="str">
-            <v>그레이스6밴</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="A28" t="str">
-            <v>그레이스
-장축6밴</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="A29" t="str">
-            <v>그레이스
-장축3밴</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="A30">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="A31" t="str">
-            <v>마이티 2.5톤</v>
-          </cell>
-        </row>
-        <row r="32">
-          <cell r="A32" t="str">
-            <v>마이티</v>
-          </cell>
-        </row>
-        <row r="33">
-          <cell r="A33" t="str">
-            <v>마이티2 터보</v>
-          </cell>
-        </row>
-        <row r="34">
-          <cell r="A34">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="35">
-          <cell r="A35">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="36">
-          <cell r="A36" t="str">
-            <v>그랜드스타렉스</v>
-          </cell>
-        </row>
-        <row r="37">
-          <cell r="A37">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="38">
-          <cell r="A38">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="39">
-          <cell r="A39">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="40">
-          <cell r="A40">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="41">
-          <cell r="A41">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="42">
-          <cell r="A42">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="43">
-          <cell r="A43">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="44">
-          <cell r="A44">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="45">
-          <cell r="A45">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="46">
-          <cell r="A46">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="47">
-          <cell r="A47">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="48">
-          <cell r="A48">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="49">
-          <cell r="A49">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="50">
-          <cell r="A50" t="str">
-            <v>포터초장축더블캡</v>
-          </cell>
-        </row>
-        <row r="51">
-          <cell r="A51" t="str">
-            <v>포터초장축슈퍼캡</v>
-          </cell>
-        </row>
-        <row r="52">
-          <cell r="A52">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="53">
-          <cell r="A53" t="str">
-            <v>포터</v>
-          </cell>
-        </row>
-        <row r="54">
-          <cell r="A54" t="str">
-            <v>포터장축켑</v>
-          </cell>
-        </row>
-        <row r="55">
-          <cell r="A55" t="str">
-            <v>포터초장축</v>
-          </cell>
-        </row>
-        <row r="56">
-          <cell r="A56" t="str">
-            <v>포터2</v>
-          </cell>
-        </row>
-        <row r="57">
-          <cell r="A57">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="58">
-          <cell r="A58" t="str">
-            <v>포터2내장탑</v>
-          </cell>
-        </row>
-        <row r="59">
-          <cell r="A59" t="str">
-            <v>포터2냉동탑</v>
-          </cell>
-        </row>
-        <row r="60">
-          <cell r="A60">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="61">
-          <cell r="A61">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="62">
-          <cell r="A62">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="63">
-          <cell r="A63">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="64">
-          <cell r="A64" t="str">
-            <v>현대5톤트럭</v>
-          </cell>
-        </row>
-        <row r="65">
-          <cell r="A65">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="66">
-          <cell r="A66">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="67">
-          <cell r="A67" t="str">
-            <v>스타렉스</v>
-          </cell>
-        </row>
-        <row r="68">
-          <cell r="A68" t="str">
-            <v>스타렉스인터쿨러9</v>
-          </cell>
-        </row>
-        <row r="69">
-          <cell r="A69" t="str">
-            <v>스타렉스9</v>
-          </cell>
-        </row>
-        <row r="70">
-          <cell r="A70">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="71">
-          <cell r="A71" t="str">
-            <v>스타렉스12</v>
-          </cell>
-        </row>
-        <row r="72">
-          <cell r="A72">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="73">
-          <cell r="A73" t="str">
-            <v>스타렉스6</v>
-          </cell>
-        </row>
-        <row r="74">
-          <cell r="A74">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="75">
-          <cell r="A75" t="str">
-            <v>스타렉스터보롱12</v>
-          </cell>
-        </row>
-        <row r="76">
-          <cell r="A76" t="str">
-            <v>스타렉스4륜</v>
-          </cell>
-        </row>
-        <row r="77">
-          <cell r="A77">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="78">
-          <cell r="A78" t="str">
-            <v>테라칸</v>
-          </cell>
-        </row>
-        <row r="79">
-          <cell r="A79">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="80">
-          <cell r="A80" t="str">
-            <v>베르나</v>
-          </cell>
-        </row>
-        <row r="81">
-          <cell r="A81" t="str">
-            <v>뉴베르나</v>
-          </cell>
-        </row>
-        <row r="82">
-          <cell r="A82" t="str">
-            <v>베르나하이브리드</v>
-          </cell>
-        </row>
-        <row r="83">
-          <cell r="A83">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="84">
-          <cell r="A84" t="str">
-            <v>카운티</v>
-          </cell>
-        </row>
-        <row r="85">
-          <cell r="A85" t="str">
-            <v>이-카운티</v>
-          </cell>
-        </row>
-        <row r="86">
-          <cell r="A86" t="str">
-            <v>벨로스터</v>
-          </cell>
-        </row>
-        <row r="87">
-          <cell r="A87" t="str">
-            <v>베르나</v>
-          </cell>
-        </row>
-        <row r="88">
-          <cell r="A88" t="str">
-            <v>아토스</v>
-          </cell>
-        </row>
-        <row r="89">
-          <cell r="A89" t="str">
-            <v>라비타</v>
-          </cell>
-        </row>
-        <row r="90">
-          <cell r="A90">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="91">
-          <cell r="A91" t="str">
-            <v>투싼</v>
-          </cell>
-        </row>
-        <row r="92">
-          <cell r="A92" t="str">
-            <v>투스카니</v>
-          </cell>
-        </row>
-        <row r="93">
-          <cell r="A93" t="str">
-            <v>티뷰론터뷸런스</v>
-          </cell>
-        </row>
-        <row r="94">
-          <cell r="A94">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="95">
-          <cell r="A95" t="str">
-            <v>쏘나타</v>
-          </cell>
-        </row>
-        <row r="96">
-          <cell r="A96" t="str">
-            <v>ef쏘나타</v>
-          </cell>
-        </row>
-        <row r="97">
-          <cell r="A97">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="98">
-          <cell r="A98" t="str">
-            <v>뉴EF쏘나타</v>
-          </cell>
-        </row>
-        <row r="99">
-          <cell r="A99" t="str">
-            <v>뉴EF쏘나타골드</v>
-          </cell>
-        </row>
-        <row r="100">
-          <cell r="A100" t="str">
-            <v>쏘나타 하이브리드</v>
-          </cell>
-        </row>
-        <row r="101">
-          <cell r="A101">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="102">
-          <cell r="A102" t="str">
-            <v>에쿠스</v>
-          </cell>
-        </row>
-        <row r="103">
-          <cell r="A103" t="str">
-            <v>i30</v>
-          </cell>
-        </row>
-        <row r="104">
-          <cell r="A104">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="105">
-          <cell r="A105" t="str">
-            <v>싼타페</v>
-          </cell>
-        </row>
-        <row r="106">
-          <cell r="A106" t="str">
-            <v>그랜저</v>
-          </cell>
-        </row>
-        <row r="107">
-          <cell r="A107" t="str">
-            <v>그랜저XG</v>
-          </cell>
-        </row>
-        <row r="108">
-          <cell r="A108" t="str">
-            <v>뉴그랜저XG</v>
-          </cell>
-        </row>
-        <row r="109">
-          <cell r="A109" t="str">
-            <v>그랜저TG</v>
-          </cell>
-        </row>
-        <row r="110">
-          <cell r="A110" t="str">
-            <v>로체</v>
-          </cell>
-        </row>
-        <row r="111">
-          <cell r="A111" t="str">
-            <v>포르테</v>
-          </cell>
-        </row>
-        <row r="112">
-          <cell r="A112" t="str">
-            <v>포르테쿱</v>
-          </cell>
-        </row>
-        <row r="113">
-          <cell r="A113" t="str">
-            <v>봉고</v>
-          </cell>
-        </row>
-        <row r="114">
-          <cell r="A114">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="115">
-          <cell r="A115" t="str">
-            <v>델타</v>
-          </cell>
-        </row>
-        <row r="116">
-          <cell r="A116" t="str">
-            <v>아벨라</v>
-          </cell>
-        </row>
-        <row r="117">
-          <cell r="A117" t="str">
-            <v>쎄라토</v>
-          </cell>
-        </row>
-        <row r="118">
-          <cell r="A118" t="str">
-            <v>k5</v>
-          </cell>
-        </row>
-        <row r="119">
-          <cell r="A119" t="str">
-            <v>k5 하이브리드</v>
-          </cell>
-        </row>
-        <row r="120">
-          <cell r="A120" t="str">
-            <v>리오</v>
-          </cell>
-        </row>
-        <row r="121">
-          <cell r="A121" t="str">
-            <v>리오RX-V</v>
-          </cell>
-        </row>
-        <row r="122">
-          <cell r="A122" t="str">
-            <v>리오sf</v>
-          </cell>
-        </row>
-        <row r="123">
-          <cell r="A123" t="str">
-            <v>세피아</v>
-          </cell>
-        </row>
-        <row r="124">
-          <cell r="A124" t="str">
-            <v>세피아2</v>
-          </cell>
-        </row>
-        <row r="125">
-          <cell r="A125" t="str">
-            <v>세피아오토</v>
-          </cell>
-        </row>
-        <row r="126">
-          <cell r="A126" t="str">
-            <v>스펙트라</v>
-          </cell>
-        </row>
-        <row r="127">
-          <cell r="A127" t="str">
-            <v>스펙트라윙</v>
-          </cell>
-        </row>
-        <row r="128">
-          <cell r="A128" t="str">
-            <v>비스토</v>
-          </cell>
-        </row>
-        <row r="129">
-          <cell r="A129" t="str">
-            <v>슈마</v>
-          </cell>
-        </row>
-        <row r="130">
-          <cell r="A130" t="str">
-            <v>프라이드웨곤</v>
-          </cell>
-        </row>
-        <row r="131">
-          <cell r="A131" t="str">
-            <v>프라이드</v>
-          </cell>
-        </row>
-        <row r="132">
-          <cell r="A132">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="133">
-          <cell r="A133" t="str">
-            <v>프런티어</v>
-          </cell>
-        </row>
-        <row r="134">
-          <cell r="A134">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="135">
-          <cell r="A135" t="str">
-            <v>스포티지</v>
-          </cell>
-        </row>
-        <row r="137">
-          <cell r="A137" t="str">
-            <v>프런티어1.3톤</v>
-          </cell>
-        </row>
-        <row r="138">
-          <cell r="A138" t="str">
-            <v>오텍봉고킹캡</v>
-          </cell>
-        </row>
-        <row r="139">
-          <cell r="A139">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="140">
-          <cell r="A140" t="str">
-            <v>프런티어1.4톤</v>
-          </cell>
-        </row>
-        <row r="141">
-          <cell r="A141" t="str">
-            <v>봉고킹캡</v>
-          </cell>
-        </row>
-        <row r="142">
-          <cell r="A142">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="143">
-          <cell r="A143" t="str">
-            <v>오텍프런티어</v>
-          </cell>
-        </row>
-        <row r="144">
-          <cell r="A144">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="145">
-          <cell r="A145" t="str">
-            <v>봉고3</v>
-          </cell>
-        </row>
-        <row r="146">
-          <cell r="A146" t="str">
-            <v>봉고3 1.2</v>
-          </cell>
-        </row>
-        <row r="147">
-          <cell r="A147" t="str">
-            <v>봉고3 1.4</v>
-          </cell>
-        </row>
-        <row r="148">
-          <cell r="A148" t="str">
-            <v>봉고3 1톤</v>
-          </cell>
-        </row>
-        <row r="149">
-          <cell r="A149" t="str">
-            <v>봉고3 카고</v>
-          </cell>
-        </row>
-        <row r="150">
-          <cell r="A150" t="str">
-            <v>봉고3 플러스</v>
-          </cell>
-        </row>
-        <row r="151">
-          <cell r="A151" t="str">
-            <v>봉고프런티어킹캡</v>
-          </cell>
-        </row>
-        <row r="152">
-          <cell r="A152" t="str">
-            <v>봉고프런티어4륜</v>
-          </cell>
-        </row>
-        <row r="153">
-          <cell r="A153" t="str">
-            <v>봉고프런티어</v>
-          </cell>
-        </row>
-        <row r="154">
-          <cell r="A154" t="str">
-            <v>봉고3 탑</v>
-          </cell>
-        </row>
-        <row r="155">
-          <cell r="A155" t="str">
-            <v>봉고 트런티어 탑</v>
-          </cell>
-        </row>
-        <row r="156">
-          <cell r="A156" t="str">
-            <v>봉고프런티어 GLS</v>
-          </cell>
-        </row>
-        <row r="157">
-          <cell r="A157" t="str">
-            <v>마티즈</v>
-          </cell>
-        </row>
-        <row r="158">
-          <cell r="A158" t="str">
-            <v>마티즈0.8at</v>
-          </cell>
-        </row>
-        <row r="159">
-          <cell r="A159" t="str">
-            <v>마티즈0.8mt</v>
-          </cell>
-        </row>
-        <row r="160">
-          <cell r="A160" t="str">
-            <v>마티즈밴 AT</v>
-          </cell>
-        </row>
-        <row r="161">
-          <cell r="A161">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="162">
-          <cell r="A162" t="str">
-            <v>윈스톰</v>
-          </cell>
-        </row>
-        <row r="163">
-          <cell r="A163" t="str">
-            <v>라노스1.3</v>
-          </cell>
-        </row>
-        <row r="164">
-          <cell r="A164" t="str">
-            <v>라노스1.5</v>
-          </cell>
-        </row>
-        <row r="165">
-          <cell r="A165" t="str">
-            <v>라노스해치백1.3</v>
-          </cell>
-        </row>
-        <row r="166">
-          <cell r="A166" t="str">
-            <v>라노스해치백1.5</v>
-          </cell>
-        </row>
-        <row r="167">
-          <cell r="A167" t="str">
-            <v>라노스</v>
-          </cell>
-        </row>
-        <row r="168">
-          <cell r="A168">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="169">
-          <cell r="A169" t="str">
-            <v>매그너스</v>
-          </cell>
-        </row>
-        <row r="170">
-          <cell r="A170">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="171">
-          <cell r="A171" t="str">
-            <v>누비라1.5</v>
-          </cell>
-        </row>
-        <row r="173">
-          <cell r="A173" t="str">
-            <v>라세티1.6</v>
-          </cell>
-        </row>
-        <row r="174">
-          <cell r="A174">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="175">
-          <cell r="A175">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="176">
-          <cell r="A176" t="str">
-            <v>라세티5</v>
-          </cell>
-        </row>
-        <row r="177">
-          <cell r="A177" t="str">
-            <v>라세티5 mt</v>
-          </cell>
-        </row>
-        <row r="178">
-          <cell r="A178">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="179">
-          <cell r="A179" t="str">
-            <v>라세티1.5</v>
-          </cell>
-        </row>
-        <row r="180">
-          <cell r="A180">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="181">
-          <cell r="A181" t="str">
-            <v>젠트라1.5</v>
-          </cell>
-        </row>
-        <row r="182">
-          <cell r="A182" t="str">
-            <v>젠트라1.6</v>
-          </cell>
-        </row>
-        <row r="183">
-          <cell r="A183" t="str">
-            <v>젠트라1.2</v>
-          </cell>
-        </row>
-        <row r="185">
-          <cell r="A185" t="str">
-            <v>칼로스1.2</v>
-          </cell>
-        </row>
-        <row r="186">
-          <cell r="A186" t="str">
-            <v>칼로스1.5</v>
-          </cell>
-        </row>
-        <row r="187">
-          <cell r="A187" t="str">
-            <v>티코</v>
-          </cell>
-        </row>
-        <row r="188">
-          <cell r="A188" t="str">
-            <v>다마스</v>
-          </cell>
-        </row>
-        <row r="189">
-          <cell r="A189" t="str">
-            <v>다마스밴</v>
-          </cell>
-        </row>
-        <row r="190">
-          <cell r="A190" t="str">
-            <v>다마스5</v>
-          </cell>
-        </row>
-        <row r="191">
-          <cell r="A191" t="str">
-            <v>다마스7</v>
-          </cell>
-        </row>
-        <row r="192">
-          <cell r="A192" t="str">
-            <v>레간자</v>
-          </cell>
-        </row>
-        <row r="193">
-          <cell r="A193" t="str">
-            <v>레간자2.0</v>
-          </cell>
-        </row>
-        <row r="194">
-          <cell r="A194" t="str">
-            <v>라보</v>
-          </cell>
-        </row>
-        <row r="195">
-          <cell r="A195" t="str">
-            <v>라보롱카고</v>
-          </cell>
-        </row>
-        <row r="196">
-          <cell r="A196">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="197">
-          <cell r="A197" t="str">
-            <v>라보5MT</v>
-          </cell>
-        </row>
-        <row r="198">
-          <cell r="A198" t="str">
-            <v>CR-V</v>
-          </cell>
-        </row>
-        <row r="199">
-          <cell r="A199" t="str">
-            <v>쏘울</v>
-          </cell>
-        </row>
-        <row r="200">
-          <cell r="A200" t="str">
-            <v>모닝</v>
-          </cell>
-        </row>
-        <row r="201">
-          <cell r="A201" t="str">
-            <v>쏘렌토</v>
-          </cell>
-        </row>
-        <row r="202">
-          <cell r="A202" t="str">
-            <v>쏘렌토gl</v>
-          </cell>
-        </row>
-        <row r="203">
-          <cell r="A203" t="str">
-            <v>쏘렌토GLS</v>
-          </cell>
-        </row>
-        <row r="204">
-          <cell r="A204">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="205">
-          <cell r="A205" t="str">
-            <v>파맥스</v>
-          </cell>
-        </row>
-        <row r="206">
-          <cell r="A206" t="str">
-            <v>타우너</v>
-          </cell>
-        </row>
-        <row r="207">
-          <cell r="A207" t="str">
-            <v>프레지오</v>
-          </cell>
-        </row>
-        <row r="208">
-          <cell r="A208">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="209">
-          <cell r="A209">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="210">
-          <cell r="A210">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="211">
-          <cell r="A211">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="212">
-          <cell r="A212" t="str">
-            <v>오피러스</v>
-          </cell>
-        </row>
-        <row r="213">
-          <cell r="A213" t="str">
-            <v>옵티마</v>
-          </cell>
-        </row>
-        <row r="214">
-          <cell r="A214" t="str">
-            <v>옵티마리갈</v>
-          </cell>
-        </row>
-        <row r="215">
-          <cell r="A215" t="str">
-            <v>sm3</v>
-          </cell>
-        </row>
-        <row r="216">
-          <cell r="A216">
-            <v>520</v>
-          </cell>
-        </row>
-        <row r="217">
-          <cell r="A217" t="str">
-            <v>520 LPG</v>
-          </cell>
-        </row>
-        <row r="218">
-          <cell r="A218">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="219">
-          <cell r="A219" t="str">
-            <v>525V</v>
-          </cell>
-        </row>
-        <row r="220">
-          <cell r="A220" t="str">
-            <v>520v</v>
-          </cell>
-        </row>
-        <row r="221">
-          <cell r="A221">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="222">
-          <cell r="A222" t="str">
-            <v>시에로</v>
-          </cell>
-        </row>
-        <row r="223">
-          <cell r="A223">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="224">
-          <cell r="A224">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="225">
-          <cell r="A225">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="226">
-          <cell r="A226">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="227">
-          <cell r="A227">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="228">
-          <cell r="A228">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="229">
-          <cell r="A229" t="str">
-            <v>bmw525i</v>
-          </cell>
-        </row>
-        <row r="230">
-          <cell r="A230">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="231">
-          <cell r="A231">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="232">
-          <cell r="A232">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="233">
-          <cell r="A233">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="234">
-          <cell r="A234">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="235">
-          <cell r="A235" t="str">
-            <v>무쏘</v>
-          </cell>
-        </row>
-        <row r="236">
-          <cell r="A236" t="str">
-            <v>뉴무쏘</v>
-          </cell>
-        </row>
-        <row r="237">
-          <cell r="A237" t="str">
-            <v>카니발</v>
-          </cell>
-        </row>
-        <row r="238">
-          <cell r="A238" t="str">
-            <v>카니발2</v>
-          </cell>
-        </row>
-        <row r="239">
-          <cell r="A239" t="str">
-            <v>카렌스</v>
-          </cell>
-        </row>
-        <row r="240">
-          <cell r="A240" t="str">
-            <v>렉스턴</v>
-          </cell>
-        </row>
-        <row r="241">
-          <cell r="A241" t="str">
-            <v>체어맨</v>
-          </cell>
-        </row>
-        <row r="242">
-          <cell r="A242">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="243">
-          <cell r="A243">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="244">
-          <cell r="A244" t="str">
-            <v>이스타나</v>
-          </cell>
-        </row>
-        <row r="245">
-          <cell r="A245" t="str">
-            <v>이스타나15</v>
-          </cell>
-        </row>
-        <row r="246">
-          <cell r="A246" t="str">
-            <v>이스타나12</v>
-          </cell>
-        </row>
-        <row r="247">
-          <cell r="A247" t="str">
-            <v>이스타나6밴</v>
-          </cell>
-        </row>
-        <row r="248">
-          <cell r="A248" t="str">
-            <v>엑티언</v>
-          </cell>
-        </row>
-        <row r="249">
-          <cell r="A249" t="str">
-            <v>엑티언스포츠</v>
-          </cell>
-        </row>
-        <row r="250">
-          <cell r="A250" t="str">
-            <v>코란도</v>
-          </cell>
-        </row>
-        <row r="251">
-          <cell r="A251" t="str">
-            <v>렉서스ES330</v>
-          </cell>
-        </row>
-        <row r="252">
-          <cell r="A252" t="str">
-            <v>렉서스ES350</v>
-          </cell>
-        </row>
-        <row r="253">
-          <cell r="A253" t="str">
-            <v>렉서스LS430</v>
-          </cell>
-        </row>
-        <row r="254">
-          <cell r="A254" t="str">
-            <v>렉서스GS300</v>
-          </cell>
-        </row>
-        <row r="255">
-          <cell r="A255" t="str">
-            <v>렉서스LS460</v>
-          </cell>
-        </row>
-        <row r="256">
-          <cell r="A256" t="str">
-            <v>렉서스LS460L</v>
-          </cell>
-        </row>
-        <row r="257">
-          <cell r="A257" t="str">
-            <v>벤츠 C-240</v>
-          </cell>
-        </row>
-        <row r="258">
-          <cell r="A258" t="str">
-            <v>아우디a6</v>
-          </cell>
-        </row>
-        <row r="259">
-          <cell r="A259" t="str">
-            <v>아우디a4</v>
-          </cell>
-        </row>
-        <row r="260">
-          <cell r="A260" t="str">
-            <v>엑센트</v>
-          </cell>
-        </row>
-        <row r="261">
-          <cell r="A261" t="str">
-            <v>스타렉스인터쿨러9인4WD</v>
-          </cell>
-        </row>
-        <row r="262">
-          <cell r="A262" t="str">
-            <v>스타렉스9</v>
-          </cell>
-        </row>
-        <row r="263">
-          <cell r="A263" t="str">
-            <v>뉴스타렉스4륜AT</v>
-          </cell>
-        </row>
-        <row r="264">
-          <cell r="A264" t="str">
-            <v>스타렉스인터쿨러단축9인</v>
-          </cell>
-        </row>
-        <row r="265">
-          <cell r="A265" t="str">
-            <v>프라이드해치백</v>
-          </cell>
-        </row>
-        <row r="266">
-          <cell r="A266" t="str">
-            <v>싼타페AT</v>
-          </cell>
-        </row>
-        <row r="267">
-          <cell r="A267" t="str">
-            <v>뉴스타렉스12</v>
-          </cell>
-        </row>
-        <row r="268">
-          <cell r="A268" t="str">
-            <v>포터II냉동탑차</v>
-          </cell>
-        </row>
-        <row r="269">
-          <cell r="A269" t="str">
-            <v>포터II슈퍼캡냉동탑차</v>
-          </cell>
-        </row>
-        <row r="270">
-          <cell r="A270" t="str">
-            <v>다마스5인승</v>
-          </cell>
-        </row>
-        <row r="271">
-          <cell r="A271" t="str">
-            <v>카운티25</v>
-          </cell>
-        </row>
-        <row r="272">
-          <cell r="A272" t="str">
-            <v>프라이드가솔린해치</v>
-          </cell>
-        </row>
-        <row r="273">
-          <cell r="A273" t="str">
-            <v>봉고 III 코치15</v>
-          </cell>
-        </row>
-        <row r="274">
-          <cell r="A274" t="str">
-            <v>그레이스15인승</v>
-          </cell>
-        </row>
-        <row r="275">
-          <cell r="A275" t="str">
-            <v>프라이드해치백디젤</v>
-          </cell>
-        </row>
-        <row r="276">
-          <cell r="A276" t="str">
-            <v>올뉴마티즈</v>
-          </cell>
-        </row>
-        <row r="277">
-          <cell r="A277" t="str">
-            <v>갤로퍼</v>
-          </cell>
-        </row>
-        <row r="278">
-          <cell r="A278" t="str">
-            <v>그랜드스타렉스12</v>
-          </cell>
-        </row>
-        <row r="279">
-          <cell r="A279" t="str">
-            <v>투싼 AT</v>
-          </cell>
-        </row>
-        <row r="280">
-          <cell r="A280" t="str">
-            <v>봉고 III 1.2톤카고</v>
-          </cell>
-        </row>
-        <row r="281">
-          <cell r="A281" t="str">
-            <v>투싼 CRDI</v>
-          </cell>
-        </row>
-        <row r="282">
-          <cell r="A282" t="str">
-            <v>카운티25</v>
-          </cell>
-        </row>
-        <row r="283">
-          <cell r="A283" t="str">
-            <v>그레이스터보15인</v>
-          </cell>
-        </row>
-        <row r="284">
-          <cell r="A284" t="str">
-            <v>그레이스터보15인승</v>
-          </cell>
-        </row>
-        <row r="285">
-          <cell r="A285" t="str">
-            <v>포터II냉동탑차</v>
-          </cell>
-        </row>
-        <row r="286">
-          <cell r="A286" t="str">
-            <v>봉고 III 코치15</v>
-          </cell>
-        </row>
-        <row r="287">
-          <cell r="A287" t="str">
-            <v>봉고 III 1톤카고</v>
-          </cell>
-        </row>
-        <row r="288">
-          <cell r="A288" t="str">
-            <v>봉고III 코치</v>
-          </cell>
-        </row>
-        <row r="289">
-          <cell r="A289" t="str">
-            <v>봉고III 1톤</v>
-          </cell>
-        </row>
-        <row r="290">
-          <cell r="A290" t="str">
-            <v>봉고 III 12인승</v>
-          </cell>
-        </row>
-        <row r="291">
-          <cell r="A291" t="str">
-            <v>오텍파라메딕특수구급차</v>
-          </cell>
-        </row>
-        <row r="292">
-          <cell r="A292" t="str">
-            <v>봉고 III 카고</v>
-          </cell>
-        </row>
-        <row r="293">
-          <cell r="A293" t="str">
-            <v>스타렉스4wdAT</v>
-          </cell>
-        </row>
-        <row r="294">
-          <cell r="A294" t="str">
-            <v>포터II 카고</v>
-          </cell>
-        </row>
-        <row r="295">
-          <cell r="A295" t="str">
-            <v>프라이드1.6</v>
-          </cell>
-        </row>
-        <row r="296">
-          <cell r="A296" t="str">
-            <v>스타렉스7인승</v>
-          </cell>
-        </row>
-        <row r="297">
-          <cell r="A297" t="str">
-            <v>뉴스타렉스9</v>
-          </cell>
-        </row>
-        <row r="298">
-          <cell r="A298" t="str">
-            <v>봉고III냉탑</v>
-          </cell>
-        </row>
-        <row r="299">
-          <cell r="A299" t="str">
-            <v>프라이드해치백디젤</v>
-          </cell>
-        </row>
-        <row r="300">
-          <cell r="A300" t="str">
-            <v>테라칸ex</v>
-          </cell>
-        </row>
-        <row r="301">
-          <cell r="A301" t="str">
-            <v>라세티</v>
-          </cell>
-        </row>
-        <row r="302">
-          <cell r="A302" t="str">
-            <v>뉴스타렉스12</v>
-          </cell>
-        </row>
-        <row r="303">
-          <cell r="A303" t="str">
-            <v>봉고III코치</v>
-          </cell>
-        </row>
-        <row r="304">
-          <cell r="A304" t="str">
-            <v>뉴스타렉스</v>
-          </cell>
-        </row>
-        <row r="305">
-          <cell r="A305" t="str">
-            <v>테라칸 JX250</v>
-          </cell>
-        </row>
-        <row r="306">
-          <cell r="A306" t="str">
-            <v>스타렉스4륜</v>
-          </cell>
-        </row>
-        <row r="307">
-          <cell r="A307" t="str">
-            <v>뉴스타렉스사륜</v>
-          </cell>
-        </row>
-        <row r="308">
-          <cell r="A308" t="str">
-            <v>라세티해치백가솔린</v>
-          </cell>
-        </row>
-        <row r="309">
-          <cell r="A309" t="str">
-            <v>스타렉스사륜</v>
-          </cell>
-        </row>
-        <row r="310">
-          <cell r="A310" t="str">
-            <v>갤로퍼II승합</v>
-          </cell>
-        </row>
-        <row r="311">
-          <cell r="A311" t="str">
-            <v>갤로퍼</v>
-          </cell>
-        </row>
-        <row r="312">
-          <cell r="A312" t="str">
-            <v>라세티해치백</v>
-          </cell>
-        </row>
-        <row r="313">
-          <cell r="A313" t="str">
-            <v>뉴스타렉스12인승2륜</v>
-          </cell>
-        </row>
-        <row r="314">
-          <cell r="A314">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="315">
-          <cell r="A315">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="316">
-          <cell r="A316">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="317">
-          <cell r="A317">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="318">
-          <cell r="A318">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="319">
-          <cell r="A319">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="320">
-          <cell r="A320">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="321">
-          <cell r="A321">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="322">
-          <cell r="A322">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="323">
-          <cell r="A323">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="324">
-          <cell r="A324">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="325">
-          <cell r="A325">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="326">
-          <cell r="A326">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="327">
-          <cell r="A327">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="328">
-          <cell r="A328">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="329">
-          <cell r="A329">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="330">
-          <cell r="A330">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="331">
-          <cell r="A331">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="332">
-          <cell r="A332">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="333">
-          <cell r="A333">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="334">
-          <cell r="A334">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="335">
-          <cell r="A335">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="336">
-          <cell r="A336">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="337">
-          <cell r="A337">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="338">
-          <cell r="A338">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="339">
-          <cell r="A339">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="340">
-          <cell r="A340">
-            <v>518</v>
-          </cell>
-        </row>
-        <row r="341">
-          <cell r="A341">
-            <v>518</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6">
-        <row r="2">
-          <cell r="G2" t="str">
-            <v>KJ1705-22</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-      <sheetData sheetId="21"/>
-      <sheetData sheetId="22"/>
-      <sheetData sheetId="23"/>
-      <sheetData sheetId="24"/>
-      <sheetData sheetId="25"/>
-      <sheetData sheetId="26"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>